<commit_message>
Fix: Hapus kolom NIS dari semua baris kode dan database karena tidak dipakai (hanya NISN)
</commit_message>
<xml_diff>
--- a/public/template_data_siswa.xlsx
+++ b/public/template_data_siswa.xlsx
@@ -397,89 +397,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>NIS</v>
+        <v>NISN</v>
       </c>
       <c r="B1" t="str">
-        <v>NISN</v>
+        <v>Nama Lengkap</v>
       </c>
       <c r="C1" t="str">
-        <v>Nama Lengkap</v>
+        <v>Kelas / Jurusan</v>
       </c>
       <c r="D1" t="str">
-        <v>Kelas / Jurusan</v>
+        <v>Tempat Lahir</v>
       </c>
       <c r="E1" t="str">
-        <v>Tempat Lahir</v>
+        <v>Tanggal Lahir</v>
       </c>
       <c r="F1" t="str">
-        <v>Tanggal Lahir</v>
+        <v>Ruang Ujian</v>
       </c>
       <c r="G1" t="str">
-        <v>Ruang Ujian</v>
-      </c>
-      <c r="H1" t="str">
         <v>Password Ujian</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1001</v>
+        <v>1234567890</v>
       </c>
       <c r="B2" t="str">
-        <v>1234567890</v>
+        <v>Ahmad Fauzan TEST</v>
       </c>
       <c r="C2" t="str">
-        <v>Ahmad Fauzan TEST</v>
+        <v>X PPLG 1</v>
       </c>
       <c r="D2" t="str">
-        <v>X PPLG 1</v>
+        <v>Jakarta</v>
       </c>
       <c r="E2" t="str">
-        <v>Jakarta</v>
+        <v>2005-08-11</v>
       </c>
       <c r="F2" t="str">
-        <v>2005-08-11</v>
+        <v>Lembar 1</v>
       </c>
       <c r="G2" t="str">
-        <v>Lembar 1</v>
-      </c>
-      <c r="H2" t="str">
         <v>123456</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1002</v>
+        <v>0987654321</v>
       </c>
       <c r="B3" t="str">
-        <v>0987654321</v>
+        <v>Budi Santoso TEST</v>
       </c>
       <c r="C3" t="str">
-        <v>Budi Santoso TEST</v>
+        <v>X PPLG 1</v>
       </c>
       <c r="D3" t="str">
-        <v>X PPLG 1</v>
+        <v>Bandung</v>
       </c>
       <c r="E3" t="str">
-        <v>Bandung</v>
+        <v>2006-02-20</v>
       </c>
       <c r="F3" t="str">
-        <v>2006-02-20</v>
+        <v>Lembar 1</v>
       </c>
       <c r="G3" t="str">
-        <v>Lembar 1</v>
-      </c>
-      <c r="H3" t="str">
         <v>654321</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>